<commit_message>
Expand golden set and improve recursive search prompt
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/golden_20260411_v1.xlsx
+++ b/tamu_data/evals/golden_sets/golden_20260411_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,11 @@
       <c r="Q1" t="inlineStr">
         <is>
           <t>run:verify_pipeline</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>run:new_golden_rows</t>
         </is>
       </c>
     </row>
@@ -609,6 +614,15 @@
 *   **Week 4 (Feb 2):** The TLB, Paging on the x86, Segmentation, Beyond Physical Memory, and Virtual Memory Mechanisms [Source 3].</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>CSCE 611, Section 600, covers the following topics in the beginning of the Spring 2026 semester:
+*   **Week 1 (Jan 12):** Project Setup, Introduction to Operating Systems, Architectural Support, and OS Structures [Source 3].
+*   **Week 2 (Jan 19):** System Calls, and Interrupts and Exceptions on the x86 [Source 3].
+*   **Week 3 (Jan 26):** Memory Allocation, Address Spaces, Paging, and Advanced Paging [Source 3].
+*   **Week 4 (Feb 2):** The TLB, Paging on the x86, Segmentation, Beyond Physical Memory, and Virtual Memory Mechanisms [Source 3].</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -700,6 +714,15 @@
         </is>
       </c>
       <c r="Q3" t="inlineStr">
+        <is>
+          <t>Upon completion of CSCE 669, students will be able to:
+*   Master basic theories and techniques in current research in computational optimization [Source 1, 2].
+*   Apply theories and techniques studied in the course to solve real-world problems in computational optimization [Source 1, 2].
+*   Use appropriate technologies to communicate, collaborate, and conduct research in the area of computational optimization [Source 2].
+*   Gain a solid background and preparation for advanced research in computational optimization and other related research areas [Source 2].</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>Upon completion of CSCE 669, students will be able to:
 *   Master basic theories and techniques in current research in computational optimization [Source 1, 2].
@@ -810,6 +833,17 @@
         </is>
       </c>
       <c r="Q4" t="inlineStr">
+        <is>
+          <t>CSCE 665 (Section 600) will introduce various modern topics in computer and network security, which may include but are not limited to:
+*   Basic network &amp; system security (e.g., software security, malware, botnet, intrusion detection) [Source 1, 2]
+*   Security in a software-defined world (e.g., SDN/NFV, Cloud, 5G/Edge, Vehicle security) [Source 2]
+*   Mobile &amp; IoT security (e.g., smartphone security, Alexa and voice app security) [Source 2]
+*   Web and Web3 security (e.g., traditional web security, spam, Web3 (DeFi, blockchain) security) [Source 2]
+*   AI/LLM security (e.g., LLM-based security, adversarial Learning / backdoor, advanced applications with AI) [Source 2]
+The tentative schedule also lists topics such as Malware Basics, Intrusion Detection, Advanced Detection &amp; Response, Software-Defined Security, Web/Web3 Security, and AI/LLM Security [Source 3].</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>CSCE 665 (Section 600) will introduce various modern topics in computer and network security, which may include but are not limited to:
 *   Basic network &amp; system security (e.g., software security, malware, botnet, intrusion detection) [Source 1, 2]
@@ -1028,6 +1062,33 @@
 Grades are assigned on a 10-point scale: 90-100 = A, 80-89 = B, 70-79 = C, 60-69 = D, and &lt;60 = F [Source 2].</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>CSCE 672, Section 600 (58439), titled "Computer Supported Collaborative Work," focuses on the design, implementation, and use of technical systems that support people working cooperatively. It draws from the research area of Computer Supported Cooperative Work (CSCW), covering current theoretical, practical, technical, and social issues, as well as future directions in the field [Source 1].
+Key topics covered in the course include:
+*   CSCW history and central issues [Source 3]
+*   Designing for artifact and human awareness [Source 3]
+*   Forms of communication [Source 3]
+*   Content sharing systems and issues [Source 3]
+*   Collaborative decision making and voting models [Source 3]
+*   Meeting capture and reuse [Source 3]
+*   Crowdsourcing and its issues [Source 3]
+*   Online communities and virtual teams [Source 3]
+*   Shared user history and its visualization [Source 3]
+*   Collaborative search and design [Source 3]
+*   Software supporting social skill development [Source 3]
+*   Collaboration in online games [Source 3]
+*   Supporting software teams [Source 3]
+To enroll, students must have completed CSCE 671 or CSCE 610, or receive approval from the instructor [Source 1].
+Your final grade will be determined by the following components:
+*   Assignment 1: 10% [Source 2]
+*   Team project: 35% [Source 2]
+*   Readings write-ups: 35% [Source 2]
+*   Readings presentations: 10% [Source 2]
+*   Attendance (via sign-in sheet): 10% [Source 2]
+Grades are assigned on a 10-point scale: 90-100 = A, 80-89 = B, 70-79 = C, 60-69 = D, and &lt;60 = F [Source 2].</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1159,6 +1220,23 @@
 The course emphasizes how humans naturally sketch, how systems interpret sketches, and how recognition algorithms behave in real-world, noisy settings. It involves hands-on implementation of recognition techniques, critical reading of research papers, in-class activities, and a semester-long team project [Source 1, 2].</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>For CSCE 624, Section 600 (58435), titled "Sketch Recognition," you should know the following before taking the course:
+**Prerequisites:**
+*   Graduate classification [Source 1, 2].
+**Recommended Knowledge:**
+*   General graduate-level knowledge in computer science [Source 2].
+*   Familiarity with at least one of the following is helpful but not strictly required:
+    *   Programming (any language) [Source 2].
+    *   Basic machine learning or artificial intelligence concepts [Source 2].
+    *   Linear algebra or probability [Source 2].
+    *   Software engineering practices [Source 2].
+*   Students from related disciplines (e.g., engineering, HCI, data science) are welcome [Source 2].
+**Course Focus:**
+The course emphasizes how humans naturally sketch, how systems interpret sketches, and how recognition algorithms behave in real-world, noisy settings. It involves hands-on implementation of recognition techniques, critical reading of research papers, in-class activities, and a semester-long team project [Source 1, 2].</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1287,6 +1365,23 @@
         </is>
       </c>
       <c r="Q7" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 638 (Section 600), "Natural Language Processing: Foundations and Techniques," would be highly beneficial for someone wanting to work with large language models (LLMs) [Source 1].
+The course directly addresses LLMs and related advanced topics, making it relevant for careers in this field. Key topics covered include:
+*   **Language Modeling** [Source 2]
+*   **Transformers** [Source 2]
+*   **Contextualized Representations, Pre-Training, Large Language Models** [Source 2]
+*   **Parameter-Efficient Fine-Tuning, Model Distillation, Evaluation** [Source 2]
+*   **Instruction Tuning, Alignment, Post-Training** [Source 2]
+*   **Large Reasoning Models, Test-Time Scaling, Decoding** [Source 2]
+*   **Retrieval-Augmented Generation, Agents** [Source 2]
+*   **Multilingual Language Models, Vision-Language Models** [Source 2]
+*   **AI-Generated Text Detection** [Source 2]
+*   **Bias Mitigation, Hallucinations** [Source 2]
+The course aims to teach Natural Language Processing (NLP) fundamentals, including language models and semantic understanding, and introduces major NLP applications [Source 1]. Upon completion, learners will be able to identify and explain fundamental NLP concepts and models, be aware of recent trends in NLP research, and apply techniques to tackle NLP challenges [Source 1, 3].</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Yes, CSCE 638 (Section 600), "Natural Language Processing: Foundations and Techniques," would be highly beneficial for someone wanting to work with large language models (LLMs) [Source 1].
 The course directly addresses LLMs and related advanced topics, making it relevant for careers in this field. Key topics covered include:
@@ -1440,6 +1535,20 @@
 While a substantial portion of the course focuses on interactive media design, you should be aware that digital rights and policy topics are also covered and are part of the learning outcomes and schedule [Source 2, 3].</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>CSCE 656: Computers and New Media (Section 600) covers a significant amount of material related to interactive media design, but also includes topics on digital rights and policy [Source 1, 2, 3, 4].
+**Academic Content Breakdown:**
+*   **Interactive Media Design Focus:**
+    *   The course investigates the impact of computers in new media design and the relationships between authors and readers of interactive materials [Source 1].
+    *   Learning outcomes include designing software features for immersion, agency, and transformation; describing techniques for creating computer characters and narrative control; developing software for audio/video manipulation; and designing, implementing, and evaluating software for content creation/consumption [Source 3].
+    *   The course schedule dedicates approximately 10 out of 14 content weeks to topics such as designing software for immersion, agency and transformation, interactive media and computer characters, interactive text and social media, bridging physical and digital media, audio/music/speech, recorded/authored video, games, and automatic narrative control [Source 2, 4].
+*   **Digital Rights and Policy Focus:**
+    *   Learning outcomes also include describing differences between physical and intellectual property, and assessing software licenses, patents, and digital rights management software [Source 3].
+    *   The course schedule dedicates approximately 4 weeks to topics like digital rights management, property rights and issues, software licenses and intellectual property, and evaluating policy effects [Source 2].
+While a substantial portion of the course focuses on interactive media design, you should be aware that digital rights and policy topics are also covered and are part of the learning outcomes and schedule [Source 2, 3].</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1577,6 +1686,22 @@
 **Prerequisites:** Graduate classification and approval of the instructor are required [Source 1, 2].</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 665, "Advanced Networking and Security," Section 600, appears to offer a strong foundation for specializing in real-world software or cloud security [Source 1].
+The course aims to provide a thorough grounding in computer and network security, suitable for students interested in real-world security issues and techniques [Source 1].
+Key topics directly relevant to your interest include:
+*   **Software security** [Source 1, 2]
+*   **Security in a software-defined world**, specifically mentioning **Cloud** security [Source 2]
+*   **Web and Web3 security** [Source 2]
+Upon completion, learners will be able to:
+*   Analyze complex trade-offs and architectural tensions in securing modern distributed systems and networks [Source 2].
+*   Synthesize fundamental security principles to design robust defenses against sophisticated threat models [Source 2].
+*   Demonstrate practical working knowledge of offensive and/or defensive techniques [Source 2].
+The course emphasizes practical application through a significant mini research project (65% of the grade), which can further enhance practical skills relevant to industry [Source 3].
+**Prerequisites:** Graduate classification and approval of the instructor are required [Source 1, 2].</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1705,6 +1830,22 @@
         </is>
       </c>
       <c r="Q10" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 641 would be a beneficial course for someone aiming for a career in game or graphics development.
+The course provides an in-depth introduction to physically based rendering, with an emphasis on Monte Carlo techniques, and covers how light interacts with objects in the real world and how image formation is mathematically formulated and solved using modern rendering algorithms [Source 1, 2].
+Key topics and skills directly relevant to game and graphics development include:
+*   **Representation of 3-dimensional objects** (polyhedral, curved surfaces, volumetric, CSG models) [Source 1]
+*   **Techniques for hidden surface/edge removal and volume rendering** [Source 1]
+*   **Illumination and shading** [Source 1]
+*   **Antialiasing, ray tracing, and radiosity** [Source 1]
+*   **Animation** [Source 1]
+*   **Practical experience with state-of-the-art graphics hardware and software** [Source 1]
+*   **Implementing core rendering algorithms** such as ray tracing, direct illumination, and global illumination methods [Source 2]
+*   **Designing and implementing a physically based rendering system or rendering component** [Source 2]
+The course focuses on both the theoretical foundations of rendering and their application in practical image synthesis systems [Source 2]. Students will gain practical experience through programming assignments in C++ and a final project where they implement additional rendering features [Source 3]. These skills are fundamental for roles in game engine development, real-time graphics, visual effects, and other areas of computer graphics.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>Yes, CSCE 641 would be a beneficial course for someone aiming for a career in game or graphics development.
 The course provides an in-depth introduction to physically based rendering, with an emphasis on Monte Carlo techniques, and covers how light interacts with objects in the real world and how image formation is mathematically formulated and solved using modern rendering algorithms [Source 1, 2].
@@ -1892,6 +2033,27 @@
 **Prerequisites:** CSCE 671 or CSCE 610 or approval of instructor [Source 1]</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 672, Computer Supported Collaborative Work, appears to be a worthwhile course if you are interested in the practical aspects of building collaborative applications.
+The course covers the "design, implementation and use of technical systems that support people working cooperatively" [Source 1]. It draws from the research area of Computer Supported Cooperative Work (CSCW) and includes current theoretical, practical, technical, and social issues [Source 1].
+Key topics covered in the course include:
+*   Designing for artifact and human awareness [Source 3]
+*   Forms of communication [Source 3]
+*   Content sharing systems and issues [Source 3]
+*   Collaborative decision making [Source 3]
+*   Collaborative search and design [Source 3]
+*   Software supporting social skill development [Source 3]
+*   Supporting software teams [Source 3]
+Upon completion, you will be able to:
+*   Prioritize issues and identify trade-offs in the design of collaborative software [Source 1, 2]
+*   Design software capabilities that facilitate awareness, communication, and coordination [Source 1, 2]
+*   Design, implement, and evaluate software to support collaboration in specific settings [Source 2]
+The course involves a team project (35% of the grade) and smaller project activities due weekly, which would provide practical experience [Source 2, 3].
+**Course ID and Section:** CSCE 672, Section 600 (58439) [Source 1]
+**Prerequisites:** CSCE 671 or CSCE 610 or approval of instructor [Source 1]</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2010,6 +2172,22 @@
         </is>
       </c>
       <c r="Q12" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 608 covers practical skills relevant to building and managing database systems in the real world. The course aims for learners to be able to develop database systems for applications, master efficient query processing techniques, and deal with system issues related to database systems [Source 2].
+Key topics covered include:
+*   Database modeling techniques [Source 1]
+*   Relational database design theory [Source 1]
+*   Query languages (including SQL) [Source 1, 3]
+*   Physical data organization [Source 1]
+*   Query processing and optimization [Source 1, 3]
+*   Transaction management and recovery [Source 1, 3]
+*   Distributed data management [Source 1]
+*   Concurrency control [Source 3]
+*   Index structures [Source 3]
+*   Bigdata [Source 3]</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
         <is>
           <t>Yes, CSCE 608 covers practical skills relevant to building and managing database systems in the real world. The course aims for learners to be able to develop database systems for applications, master efficient query processing techniques, and deal with system issues related to database systems [Source 2].
 Key topics covered include:
@@ -2182,6 +2360,31 @@
 These examples demonstrate that final grades can be influenced by various factors beyond a simple arithmetic average of all graded components.</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Yes, based on the provided course syllabi, there are several instances where a final grade is not solely determined by a straightforward calculated average of component scores. The principle at play is that grading policies can incorporate various mechanisms beyond a simple weighted average, including instructor discretion, specific passing conditions, dropping low scores, applying curves, peer evaluation multipliers, and bonus opportunities.
+Here are examples of such policies:
+*   **Instructor Discretion and Overriding Grades:**
+    *   In CSCE 632, the instructor "may assign a failing grade regardless of a student’s computed final score" if warranted [Source 3].
+    *   For CSCE 632, the instructor can also modify a peer evaluation multiplier at their discretion, which directly impacts a student's project score [Source 3].
+*   **Specific Passing Conditions:**
+    *   In CSCE 681, to pass the course, students must complete a syllabus quiz on Canvas with a 100% grade AND receive an average score of 80% or higher. Any course requirements completed before passing the syllabus quiz will not be considered [Source 8].
+*   **Dropping Lowest Grades:**
+    *   CSCE 629 drops the lowest grade in quizzes/exercises and the lowest homework grade [Source 1, 5].
+    *   CSCE 681 calculates the final quiz grade as the statistical mean of the top 75% of individual quiz grades, effectively dropping the lowest 25% [Source 4].
+*   **Curves:**
+    *   CSCE 629 states that "A slight curve might be applied if the course average is low" [Source 5].
+*   **Peer Evaluation Multipliers:**
+    *   In CSCE 632, a student's score on team projects is based on peer evaluations, and the instructor establishes a multiplier based on these evaluations, which can adjust the final project score [Source 3].
+*   **Bonus Opportunities:**
+    *   CSCE 648 mentions that students who regularly contribute insightful comments during class discussions may receive bonus points [Source 7].
+    *   CSCE 713 offers an optional "Independent-Study Reports" component that can add +10% to the total grade [Source 2].
+*   **Attendance-Based Deductions:**
+    *   CSCE 648 deducts 1.0 point from the class participation grade for each missed class, up to a maximum of 12 points [Source 7].
+*   **Completion Rate Adjustments:**
+    *   CSCE 632 calculates a completion rate for group class activities and adds 15% (capped at 100%) to the score, allowing students to miss some activities without negative impact [Source 10].</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2275,6 +2478,12 @@
 *   **Online Communities:** "week 9: online communities and virtual teams" [Source 1]
 *   **Collaboration in Games:** "week 13: collaboration in online games" [Source 1]
 I cannot find information about other courses at TAMU that cover these specific topics in the provided context.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Based on the provided context, the course CSCE 672: Computer Supported Collaborative Work explicitly covers topics such as crowdsourcing, online communities, and collaboration in online games [Source 1, Source 2].
+However, I cannot find information about *other* courses at TAMU that cover these specific topics in the provided context. I don't have enough data to answer this accurately based on the available syllabi.</t>
         </is>
       </c>
     </row>
@@ -2428,6 +2637,23 @@
     *   Focuses on "AI/LLM Security" across Weeks 11, 13, and 14 [Source 10].</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Several courses at Texas A&amp;M cover advanced topics in AI, including transformers and large language models:
+*   **CSCE 638: Natural Language Processing: Foundations and Techniques**
+    *   Week 5: Transformers [Source 1]
+    *   Week 6: Contextualized Representations, Pre-Training, Large Language Models [Source 1]
+*   **CSCE 624: Foundations of Sketch Recognition**
+    *   Weeks 8-9: Hidden Markov Models, LLMs, and related techniques [Source 5]
+*   **CSCE 670: Information Retrieval and Web Search**
+    *   Week 10: Transformer; BERT-Based Ranking [Source 2]
+    *   Week 12: Large Language Models Basics [Source 2]
+    *   Week 13: Large Language Models with Search Engines [Source 2]
+    *   Week 14: Large Language Models for Ranking and Recommendation [Source 2]
+*   **CSCE 665: Advanced Topics in Security**
+    *   Weeks 11-15: AI/LLM Security [Source 10]</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2534,6 +2760,15 @@
     *   Class participation and presentation are also components of the grade, suggesting discussion of technical content [Source 10].
     *   The course material primarily consists of various research papers from top security conferences and journals [Source 10].
 These courses explicitly involve activities such as writing reviews of research papers, leading discussions on technical articles, conducting literature reviews, and giving presentations on research topics, which directly align with the skills mentioned in your question.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>For students interested in improving their skills in preparing research reports and discussing technical articles, the following Texas A&amp;M CS courses would be beneficial:
+*   **CSCE 681 (Seminar)**: This course's primary purpose is to expose students to current and seminal research topics. Upon completion, students are expected to be able to prepare reports and discuss research works and selected published technical articles. Students are required to write a report for each lecture, which includes sections like background, problem statement, proposed solution, results, and critique [Source 1, 2].
+*   **CSCE 635**: In this course, students are expected to submit short reviews of research papers, articulating their understanding of main contributions, providing critical analysis of strengths and limitations, and discussing open research questions or potential extensions. Students also lead class discussions on assigned papers, preparing slides or discussion prompts to facilitate conversation around methodology, results, and broader implications [Source 3].
+*   **CSCE 632**: This course requires students to compile a literature review on an accessibility topic, based on at least 10 peer-reviewed conference or journal papers. The literature review must clearly lay out themes and gaps in research, supported by evidence. Students also give a "Current Research Presentation" based on their literature review [Source 9].
+*   **CSCE 665**: This course includes a "Paper mini-review" component and emphasizes "Class participation and presentation" [Source 10].</t>
         </is>
       </c>
     </row>
@@ -2705,6 +2940,33 @@
 While the provided context highlights the critical periods for assignments and the varying late work policies, it does not explicitly detail strategies for managing the end-of-semester workload. Therefore, I cannot provide specific strategies based solely on the available syllabi.</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Managing the end-of-semester workload, especially when multiple final projects and papers are due around the same time, requires proactive planning and effective time management. The principle is to anticipate peak workload periods and distribute tasks over time to avoid last-minute crunch.
+Based on the provided course schedules for the 202611 term, it is evident that many significant deliverables, such as final projects, reports, and presentations, often converge in late April and early May:
+*   **Late April:**
+    *   CSCE 632 has a Final Presentation on April 21 &amp; 23, with the Final Report and Video Demo due on April 28 [Source 3].
+    *   CSCE 635 has Final Project Presentations and Feedback on April 17, 20, 22, and the Final Project Report due on April 27 [Source 8].
+    *   CSCE 652 dedicates Weeks 14 and 15 to "FINAL PROJECT TIME," with the Final Project due on April 28 and the CTF Scoreboard closing on April 21 [Source 2].
+    *   CSCE 672 schedules Final project presentations for April 27-28 [Source 5].
+    *   CSCE 656 also has Final project presentations between April 20-28 [Source 7].
+*   **Early May:**
+    *   CSCE 611 has Machine Problem 7 (MP7) due on May 3, just before the Final Exam on May 5 [Source 1].
+    *   CSCE 633's Final Project is due on May 4 [Source 4].
+    *   CSCE 672's Final project reports are due on May 1 [Source 5].
+    *   CSCE 752 has its Final Exam on May 1 [Source 6].
+    *   CSCE 656 has a Survey paper due on May 1 and Final project reports due on May 1 [Source 7].
+Given this clustering of deadlines, here are some effective strategies for managing your end-of-semester workload:
+1.  **Early Identification of Deadlines:** At the beginning of the semester, review all syllabi to identify major project, paper, and exam dates. Create a master calendar that includes all these significant deadlines [Source 1, 2, 3, 4, 5, 6, 7, 8].
+2.  **Break Down Large Tasks:** For each final project or paper, break it down into smaller, manageable sub-tasks (e.g., research, outline, first draft, revisions). Assign mini-deadlines for these sub-tasks throughout the semester, well in advance of the final due date.
+3.  **Prioritize and Allocate Time:** Assess the weight and complexity of each final deliverable. Allocate more time to projects that are worth a higher percentage of your grade or require more intensive effort.
+4.  **Start Early:** Begin working on final projects and papers as soon as possible. For example, CSCE 672 and CSCE 656 mention smaller project activities and reading write-ups due weekly, which can help you stay engaged and prepare for larger deliverables [Source 5, 7]. CSCE 752 notes that projects are due approximately every two weeks, encouraging consistent work [Source 6].
+5.  **Utilize "Buffer" Time:** Build in extra time for unexpected challenges, technical issues, or the need for additional revisions. Some courses, like CSCE 611, explicitly state "hard" due dates for final assignments like MP7 to allow for timely grading, emphasizing the need to meet deadlines [Source 1].
+6.  **Leverage Regular Assignments:** Some courses have regular assignments (e.g., weekly machine problems in CSCE 611 [Source 1], bi-weekly projects in CSCE 752 [Source 6]) that can help you practice skills and stay on track, reducing the burden at the very end.
+**Planning Dimension:**
+Understanding this end-of-semester convergence is crucial for your academic progression. By proactively mapping out your major assignments from all courses, you can strategically distribute your workload, identify potential conflicts, and avoid overwhelming periods. This allows you to produce higher quality work, reduce stress, and ensure you meet all academic requirements effectively.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2825,6 +3087,19 @@
 While CSCE 679 explicitly requires a single, tool-specific project for 50% of the grade for graduate students, and CSCE 713 also has a single component worth 50%, this structure is not observed in all other graduate CS courses listed in the context.</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Grading policies and the weighting of assessment components, such as projects, vary across different courses. In the provided context, there are instances where a significant portion of the final grade is allocated to projects, sometimes with specific tool requirements.
+Specifically:
+*   In **CSCE 679**, the course project accounts for 50% of the final grade. Graduate students are required to implement their project using the D3.js visualization library [Source 1]. This aligns directly with your example of a single, tool-specific project counting for half the grade.
+*   In **CSCE 713**, "Vulnerabilities PoC" (Proof of Concept) is an individual component worth 50% of the grade. Students are required to deliver PoCs for vulnerabilities explained in class, which involves running security tools [Source 3]. While this is a single grading category, the description suggests it might involve multiple proofs of concept rather than one monolithic project.
+Other courses show different project weightings and structures:
+*   **CSCE 648** includes "Projects" worth 36 points out of 100, which are comprised of six equally weighted projects [Source 4, 6].
+*   **CSCE 652** has a "Final Project" worth 30% of the overall grade [Source 7].
+*   **CSCE 748** includes "Programming assignments" worth 50%, but these consist of five separate assignments, not a single project. It also has a "Final project" worth 20% [Source 9].
+Based on the available syllabi, while not every course follows this model, at least one course (CSCE 679) explicitly features a single, tool-specific project (D3.js) for graduate students that accounts for 50% of the final grade [Source 1]. Another course (CSCE 713) also has a significant individual, tool-related component ("Vulnerabilities PoC") weighted at 50% [Source 3].</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2892,6 +3167,11 @@
         </is>
       </c>
       <c r="Q19" t="inlineStr">
+        <is>
+          <t>The midterm exam for CSCE 629, Section 600, is scheduled for Thursday, February 26, in class [3].</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
         <is>
           <t>The midterm exam for CSCE 629, Section 600, is scheduled for Thursday, February 26, in class [3].</t>
         </is>
@@ -2973,6 +3253,11 @@
           <t>The required textbook for CSCE 608, Section 600, is "Database Systems: The Complete Book" by H. Garcia-Molina, J. Ullman, and J. Widom, 2nd Edition, published by Pearson Prentice Hall in 2009. The ISBN is 978-0-13-187325-4 [Source 2].</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>The required textbook for CSCE 608, Section 600, is "Database Systems: The Complete Book" by H. Garcia-Molina, J. Ullman, and J. Widom, 2nd Edition, published by Pearson Prentice Hall in 2009. The ISBN is 978-0-13-187325-4 [Source 2].</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3040,6 +3325,11 @@
         </is>
       </c>
       <c r="Q21" t="inlineStr">
+        <is>
+          <t>For CSCE 633, the permitted programming language is Python. It must be executable on CS unix hosts or other public systems in the department lab [Source 1, Source 2].</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>For CSCE 633, the permitted programming language is Python. It must be executable on CS unix hosts or other public systems in the department lab [Source 1, Source 2].</t>
         </is>
@@ -3135,6 +3425,15 @@
         </is>
       </c>
       <c r="Q22" t="inlineStr">
+        <is>
+          <t>Upon completion of CSCE 633, students are expected to be able to [Source 1, Source 2]:
+*   Formalize the fundamental techniques and methods of machine learning, including methods, data processing, and model selection.
+*   Analyze and compare the strengths and weaknesses of commonly used machine learning approaches.
+*   Evaluate the underlying mathematical relationships within and across advanced machine learning algorithms and the paradigms of supervised and unsupervised learning.
+*   Design, implement, and apply various advanced machine learning algorithms in a range of real-world applications.</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
         <is>
           <t>Upon completion of CSCE 633, students are expected to be able to [Source 1, Source 2]:
 *   Formalize the fundamental techniques and methods of machine learning, including methods, data processing, and model selection.
@@ -3252,6 +3551,18 @@
 The prerequisite for this course is CSCE 629 [Source 1]. Grading is based on homework assignments (30%), a course project (35%), and a final exam (35%) [Source 2].</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Upon completing CSCE 669, students will be able to:
+*   Master basic theories and techniques in current research in computational optimization [Source 1, 2].
+*   Apply these theories and techniques to solve real-world problems in computational optimization [Source 1, 2].
+*   Use appropriate technologies to communicate, collaborate, and conduct research in computational optimization [Source 2].
+*   Gain a solid background and preparation for advanced research in computational optimization and related areas [Source 2].
+This course, CSCE 669 Section 600, focuses on the combinatorial theory of polytopes for solving combinatorial optimization problems, including applications to max flow, matching, and matroids [Source 1]. The geometric interpretation of these results highlights the role of polyhedral combinatorics in designing and understanding the complexity of approximation algorithms [Source 1].
+**Career Relevance:** The course directly prepares students for advanced research in computational optimization, indicating its relevance for academic and R&amp;D careers. The ability to apply theories and techniques to "real-world problems" suggests its utility in industry roles that involve complex problem-solving, algorithm design, and optimization in fields like logistics, data science, machine learning, and operations research [Source 1, 2]. The course project, which involves reading recent published papers and conducting research on current problems, further enhances skills valuable for innovation and problem-solving in professional settings [Source 2].
+The prerequisite for this course is CSCE 629 [Source 1]. Grading is based on homework assignments (30%), a course project (35%), and a final exam (35%) [Source 2].</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3351,6 +3662,15 @@
 *   Demonstrate a practical working knowledge of offensive and/or defensive techniques to contextualize theoretical concepts [Source 2].</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Upon completion of CSCE 665 (Section 600), students will be able to:
+*   Analyze the complex trade-offs and architectural tensions inherent in securing modern distributed systems and networks [Source 2].
+*   Synthesize fundamental security principles and mechanisms to design robust defenses against sophisticated threat models [Source 2].
+*   Critique state-of-the-art security literature to identify open problems, methodological flaws, and emerging trends in the field [Source 2].
+*   Demonstrate a practical working knowledge of offensive and/or defensive techniques to contextualize theoretical concepts [Source 2].</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3418,6 +3738,11 @@
         </is>
       </c>
       <c r="Q25" t="inlineStr">
+        <is>
+          <t>All course information for CSCE 608, Section 600, will be posted in Canvas [Source 2]. Students should check course announcements, course material, and due dates daily [Source 2].</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
         <is>
           <t>All course information for CSCE 608, Section 600, will be posted in Canvas [Source 2]. Students should check course announcements, course material, and due dates daily [Source 2].</t>
         </is>
@@ -3508,6 +3833,13 @@
         </is>
       </c>
       <c r="Q26" t="inlineStr">
+        <is>
+          <t>Yes, the learning objectives for CSCE 681 seem attainable for preparing reports and discussing research.
+The course explicitly states that "Upon completion of the course, students should be able to prepare reports and discuss research works and selected published technical articles" [Source 1, Source 2].
+To achieve this, students in Section 600 are expected to attend all lectures and write a report for each. These reports are structured to include sections such as background, problem statement, proposed solution, results, and critique, directly supporting the development of report preparation and research discussion skills [Source 2]. Students in Section 700 also write reports for each lecture, which are in the form of quizzes related to the lecture content [Source 4].</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
         <is>
           <t>Yes, the learning objectives for CSCE 681 seem attainable for preparing reports and discussing research.
 The course explicitly states that "Upon completion of the course, students should be able to prepare reports and discuss research works and selected published technical articles" [Source 1, Source 2].
@@ -3707,6 +4039,37 @@
         </is>
       </c>
       <c r="Q27" t="inlineStr">
+        <is>
+          <t>CSCE 611, Section 600 (50668), is an Operating Systems course offered in Spring 2026 [Source 3].
+**Course Purpose:**
+This course provides an overview of the general architecture and key components of modern operating systems. Students will leverage knowledge from previous courses in Computer Architecture and Computer Systems to understand and implement aspects of operating systems, including memory management, persistent storage and file systems, threading, scheduling, and resource management. A significant component involves implementing a simple operating system capable of booting and running on a bare PC [Source 2].
+**Prerequisites:**
+CSCE 313 and graduate classification are required [Source 2, 3].
+**Grading Policy:**
+The course grading is based on the following components [Source 7]:
+*   Midterm: 200 points
+*   Final Exam: 200 points
+*   Design and Programming Assignments (Machine Problems): 400 points
+*   Daily Quizzes: 100 points
+*   Homework Assignments: 100 points
+A standard letter grading scale is used: A = 90% and above, B = 80% and above, C = 70% and above, D = 60% and above, F = less than 60% [Source 7].
+**Early Week Topics (OS Structures and Memory Management):**
+The course schedule outlines the following topics for the initial weeks [Source 1]:
+| Week | Day | Topic                                                              |
+| :--- | :-- | :----------------------------------------------------------------- |
+| 1    | Tue | Project Setup, Intro: What is an OS?                               |
+|      | Thu | Architectural Support, OS Structures                               |
+| 2    | Tue | System Calls                                                       |
+|      | Thu | Interrupts and Exceptions on the x86                               |
+| 3    | Tue | Memory: Memory Allocation, Address Spaces                          |
+|      | Thu | Paging, Advanced Paging                                            |
+| 4    | Tue | The TLB, Paging on the x86                                         |
+|      | Thu | Segmentation, Beyond Physical Memory, Virtual Memory Mechanisms    |
+| 5    | Tue | Page Replacement Policies I                                        |
+|      | Thu | Page Replacement Policies II, Recursive Page Table Lookup          |</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
         <is>
           <t>CSCE 611, Section 600 (50668), is an Operating Systems course offered in Spring 2026 [Source 3].
 **Course Purpose:**
@@ -3905,6 +4268,19 @@
 | Assignment Type | Component      | Due Date/Class Date                               | Weighting (of total grade) | Notes                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                             </t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For CSCE 670, Section 600 (46627), effective time management will be crucial due to the distribution of assignments throughout the semester [Source 4].
+Here's a breakdown of the major components and their deadlines to help you plan:
+**Grading Breakdown:**
+*   **Homeworks:** 30%
+*   **Quizzes:** 20%
+*   **Final:** 30%
+*   **Group Project:** 20% [Source 2]
+**Key Components and Dates:**
+| Assignment Type | Component      | Due Date/Class Date                               | Weighting (of total grade) | Notes                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                             </t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4108,6 +4484,46 @@
 *   **Late Work Policy**: Penalties for unexcused late submissions are 5% per calendar day, unless specified otherwise. Each student/team has a limited number of "late days" they may use by request. Work submitted as makeup for an excused absence is exempt from the late work policy [Source 7].</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>For CSCE 632, Section 600 (54784), Accessible Computing, here's an overview of the course and how final grades are determined:
+**Course Overview**
+*   **Course ID &amp; Section**: CSCE 632, Section 600 (54784) [Source 5]
+*   **Term**: Spring 2026 [Source 5]
+*   **Meeting Times**: Tuesdays and Thursdays, 12:45 PM - 2:00 PM, in ZACH 350 [Source 5]
+*   **Credit Hours**: 3 [Source 5]
+*   **Catalog Description**: This course explores traditionally disenfranchised user populations due to disability, including discrimination and population characteristics. It reviews ethical and legal motivations for creating accessible technology, universal design, and its role in the development, evaluation, design, and implementation of equitable and inclusive software and computer-based solutions. It also covers the application of accessibility standards and the compilation of a literature review on a current topic in accessible computing [Source 5].
+*   **Prerequisites**: Graduate classification [Source 5].
+**Grading Breakdown**
+The final grade for CSCE 632 is determined by the following components:
+*   **Pre-Class Engagement**: 5% [Source 1]
+    *   Includes course readings, quizzes, polls, and surveys. Credit is given for submissions prior to class. A completion rate is calculated, capped at 100% with a 15% allowance for missed engagements [Source 1].
+*   **Group Class Activities**: 10% [Source 1]
+    *   Students work in groups of at least 3. Credit is given for attending class and providing what is required for the activity. A completion rate is calculated, capped at 100% with a 15% allowance for missed activities [Source 1, 2].
+*   **Assignments**: 25% [Source 2]
+    *   Completed individually or with others. Some assignments are peer-graded, with scores based on peer evaluations and self-evaluation of other student assignments. Students can lose points for grading significantly differently than peers or giving all students the same scores [Source 2].
+*   **Quick Applications**: 20% [Source 2]
+    *   Timed assignments designed for quick application of class materials, typically taking 15-20 minutes but with at least 45 minutes provided [Source 2].
+*   **Literature Review**: 10% [Source 3]
+    *   Students compile a literature review on an accessibility topic, comprising at least 10 related peer-reviewed conference or journal papers. It must clearly lay out themes and gaps, supported by evidence, and include an annotated bibliography [Source 3].
+*   **Current Research Presentation**: 5% [Source 3]
+    *   A summary of HCI research based on the student's Literature Review. This is peer-graded, with scores based on peer evaluations and self-evaluation of other student assignments. Students can lose points for grading significantly differently than peers or giving all students the same scores [Source 3].
+*   **Team Project**: 25% [Source 3]
+    *   Students work in groups to address a barrier for people with disabilities that lacks an acceptable solution. The team's barrier must be instructor-approved. Teams design and implement a technology-based solution for equitable interactions. Parts of this are peer-graded, with scores based on peer evaluations and self-evaluation. The instructor may apply a multiplier based on team peer evaluations, which can be modified at their discretion [Source 3, 4].
+**Grading Scale**
+Grades are rounded to the nearest whole number and assigned as follows [Source 4]:
+*   **A**: ≥ 90 (Excellent)
+*   **B**: &lt; 90 and ≥ 80 (Good)
+*   **C**: &lt; 80 and ≥ 70 (Satisfactory)
+*   **D**: &lt; 70 and ≥ 60 (Passing)
+*   **F**: &lt; 60 (Failing)
+**Important Grading Policies**
+*   **Grade Auditing**: The instructor reserves the right to audit grades for any assignments, which may result in increasing or decreasing scores, even for already released grades [Source 1, 6].
+*   **Instructor Modifications**: The instructor may assign a failing grade regardless of a student’s computed final score if warranted. Failing to complete work can also lead to letter grade reductions [Source 4, 7].
+*   **Challenging Grades**: Any challenge to a grade must be made within one week of its publication [Source 1, 6].
+*   **Late Work Policy**: Penalties for unexcused late submissions are 5% per calendar day, unless specified otherwise. Each student/team has a limited number of "late days" they may use by request. Work submitted as makeup for an excused absence is exempt from the late work policy [Source 7].</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4227,6 +4643,21 @@
         </is>
       </c>
       <c r="Q30" t="inlineStr">
+        <is>
+          <t>CSCE 669, Section 600 (58438), is a Computational Optimization course offered in Spring 2026 [Source 4].
+The grading breakdown for the course is as follows:
+*   **Homework:** 30% (3 assignments, 10% each) [Source 1, 2]
+*   **Course project:** 35% [Source 1, 2]
+*   **Final exam:** 35% [Source 1, 2]
+The grading scale is:
+*   **A:** 90-100% [Source 1, 2]
+*   **B:** 70-89% [Source 1, 2]
+*   **C:** 60-70% [Source 1, 2]
+*   **F:** 0-59% [Source 1, 2]
+No late submissions will be accepted for assignments and projects, but unusual circumstances can be discussed with the instructor in advance [Source 1]. The final exam is comprehensive [Source 2].</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
         <is>
           <t>CSCE 669, Section 600 (58438), is a Computational Optimization course offered in Spring 2026 [Source 4].
 The grading breakdown for the course is as follows:
@@ -4388,6 +4819,23 @@
 The instructor for this course is Yu Zhang [Source 1].</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>CSCE 670, Section 600, "Information Storage and Retrieval," is offered in Spring 2026 [Source 1].
+**Course Purpose and Topics:**
+This course covers the representation, storage, and access to very large multimedia document collections. It focuses on the fundamental data structures and algorithms used in information storage and retrieval systems, as well as techniques for designing and evaluating complete retrieval systems. This includes algorithms for indexing, compressing, and querying large collections [Source 1].
+Key topics and algorithms covered include:
+*   **Web Search**: Text indexing, retrieval models, evaluation, Web crawling, link-based algorithms like PageRank, and learning to rank [Source 3].
+*   **Recommender Systems**: Collaborative filtering, matrix factorization, recommender system evaluation, and implicit recommendation [Source 3].
+*   **Advanced Topics**: Adversarial information retrieval, neural models of retrieval and recommendation [Source 3].
+*   **Specific Algorithms/Models**: Boolean Retrieval, TF-IDF, Vector Space Model, BM25, Link Analysis, Learning to Rank, Content-Based Recommender Systems, Collaborative Filtering, Matrix Factorization, Bayesian Personalized Ranking, word2vec, Neural Ranking, Transformer, BERT-Based Ranking, Neural Collaborative Filtering, Sequential Recommendation, and Large Language Models (basics, with search engines, and for ranking/recommendation) [Source 2].
+**Prerequisites:**
+Students must have completed CSCE 310 or CSCE 603, or have instructor approval, and be of graduate classification [Source 1, 3].
+**Grading (Late Work Policy):**
+For homework assignments, students are allotted five late days in total. A late day is an indivisible 24-hour unit. Once these five late days are used, any subsequent late assignment will receive a grade of 0 [Source 2].
+The instructor for this course is Yu Zhang [Source 1].</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4493,6 +4941,18 @@
 CSCE 665, "Advanced Networking and Security," appears to be a suitable follow-up course. Its catalog description indicates it covers "security aspects of various network protocols" and "modern topics in computer and network security" [Source 6, 7]. This directly builds upon the networking fundamentals and the "analysis of performance and security of networks" learned in CSCE 612 [Source 2].
 While the prerequisites for CSCE 665 are "Graduate classification and approval of instructor" [Source 6, 7] rather than CSCE 612 specifically, its content aligns well as a subsequent course for students interested in specializing in networking and security.
 The context does not explicitly list CSCE 612 as a prerequisite for any other course, nor does it provide a recommended course sequence for academic planning beyond the individual course descriptions.</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Academic progression often involves building upon foundational courses by taking more specialized or advanced courses in related fields. Given that CSCE 612 focuses on "Applied Networks and Distributed Processing," including "network design and protocol analysis," "computer communications," and "principles of network engineering" [Source 1], and covers analyzing the "security of networks" [Source 2], subsequent courses would typically delve deeper into advanced networking topics or specialize in network security.
+Based on the provided context, here are courses that would logically follow CSCE 612:
+*   **CSCE 665: Advanced Networking and Security**
+    *   This course directly builds upon the networking foundation of CSCE 612 by focusing on "Security aspects of various network protocols" [Source 6]. It covers modern topics such as "Basic network &amp; system security," "Security in a software-defined world," and "Web and Web3 security" [Source 7]. Taking CSCE 665 would allow you to analyze "complex trade-offs and architectural tensions inherent in securing modern distributed systems and networks" and design "robust defenses against sophisticated threat models," which aligns with and expands upon the security analysis aspect of CSCE 612 [Source 7, 2].
+*   **CSCE 713: Advanced Topics in Security**
+    *   While broader in scope, CSCE 713 includes significant "Network Security" topics, such as Man-In-The-Middle (MITM) Attacks, ARP Spoofing, Port Scanning, and Honeypots [Source 9]. This course would allow you to "perform penetration testing on previously unknown software" and "analyze existing source code for functional correctness" [Source 11], which could be a valuable specialization after understanding network fundamentals in CSCE 612.
+**Note on CSCE 611:** CSCE 611 (Operating Systems) is listed with CSCE 313 as a prerequisite, similar to CSCE 612 [Source 8, 2]. The content of CSCE 611, which covers operating system components, virtualization, and distributed systems [Source 8], is foundational and often taken *before* or *concurrently* with advanced networking courses like CSCE 612, rather than after. CSCE 612 itself mentions utilizing "operating-system sockets APIs" and building "multi-threaded decentralized frameworks" [Source 2], indicating that OS knowledge is beneficial prior to or during the course.
+I don't have enough data to provide a comprehensive list of all possible follow-up courses based on the available syllabi, but CSCE 665 and CSCE 713 are strong candidates for academic progression after CSCE 612.</t>
         </is>
       </c>
     </row>
@@ -4633,6 +5093,20 @@
 These courses offer a progression from foundational data handling and machine learning to advanced optimization, providing a comprehensive academic path for someone specializing in web search and recommender systems.</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>CSCE 670, "Information Storage and Retrieval," focuses on the representation, storage, and access of large multimedia document collections, covering fundamental data structures and algorithms for retrieval systems, including indexing, compressing, and querying. It specifically addresses web search and recommender systems, including topics like link-based algorithms (e.g., PageRank), learning to rank, collaborative filtering, matrix factorization, and neural models for retrieval and recommendation, as well as Large Language Models (LLMs) in the context of search engines and recommendation [Source 1, 2, 3].
+For a student interested in web search or recommender systems, the following courses would complement CSCE 670 well:
+*   **CSCE 638: Natural Language Processing: Foundations and Techniques**
+    *   **Principle**: Natural Language Processing (NLP) is foundational for understanding and processing textual data, which is critical for effective web search and many recommender systems.
+    *   **Application**: CSCE 638 covers NLP fundamentals, including language models, syntactic processing, semantic understanding, and applications like information extraction and text summarization [Source 6]. Its schedule includes topics such as word representations, transformers, contextualized representations, pre-training, and Large Language Models [Source 10]. These topics directly enhance the understanding of advanced techniques like "Neural Ranking," "Transformer; BERT-Based Ranking," and "Large Language Models with Search Engines" covered in CSCE 670 [Source 3]. Taking CSCE 638 would provide a deeper theoretical and practical background in the NLP techniques that power modern search and recommendation.
+*   **CSCE 676: Data Mining and Analysis**
+    *   **Principle**: Data mining provides a broad set of techniques for discovering patterns and insights from large datasets, which are essential for building and evaluating complex search and recommendation systems.
+    *   **Application**: CSCE 676 offers an overview of data mining, integrating concepts from machine learning and statistics, including exploratory data analysis, pattern mining, clustering, classification, and applications to online data [Source 8]. Specifically, its coverage of "Text Mining," "Graph Mining," and "Large-Scale ML" [Source 7, 9] directly relates to the challenges of processing and analyzing the massive datasets involved in information retrieval and recommender systems. The course also lists "Mining of Massive Data Sets" as a required textbook [Source 9], which is an optional resource for CSCE 670 [Source 2, 4], indicating a strong thematic connection. This course would provide a broader toolkit for handling and extracting value from the data that feeds into search and recommendation algorithms.
+**Academic Progression:**
+Taking CSCE 638 would deepen your understanding of the linguistic and semantic aspects crucial for advanced search and recommendation, especially with the increasing role of Large Language Models. CSCE 676 would provide a broader methodological foundation in handling and analyzing large datasets, which is vital for the scalability and effectiveness of these systems. These courses collectively offer a comprehensive skill set, moving from the core retrieval mechanisms (CSCE 670) to the underlying data processing (CSCE 676) and linguistic understanding (CSCE 638) necessary for cutting-edge web search and recommender systems.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4750,6 +5224,19 @@
 *   **CSCE 676 (Data Mining and Analysis)**: This course focuses on "data mining and analysis," including "data preparation," "normalization," and "large-scale mining" [Source 10]. While CSCE 608 is about managing data, data mining often utilizes data stored in databases, making these fields complementary. The course also uses "Mining of Massive Data Sets" as a required textbook [Source 10], which suggests a connection to large-scale data handling that can relate to distributed data management in CSCE 608.</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Based on the provided context, CSCE 670 (Information Storage and Retrieval) appears to be similar to CSCE 608 (Database Systems).
+Here's a comparison:
+*   **CSCE 608 (Database Systems)** [Source 1, 2]
+    *   **Catalog Description:** Covers database modeling techniques, query languages, data models, physical data organization, relational database design theory, query processing, transaction management, recovery, and distributed data management.
+    *   **Prerequisite:** CSCE 310 or approval of Instructor.
+*   **CSCE 670 (Information Storage and Retrieval)** [Source 5]
+    *   **Catalog Description:** Focuses on representation, storage, and access to very large multimedia document collections; fundamental data structures and algorithms of information storage and retrieval systems; techniques to design and evaluate complete retrieval systems, including algorithms for indexing, compressing, and querying very large collections.
+    *   **Prerequisites:** CSCE 310 or CSCE 603 or approval of instructor; graduate classification.
+Both courses deal with the storage, organization, retrieval, and querying of data, and both list CSCE 310 as a prerequisite [Source 1, 5].</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4866,6 +5353,13 @@
 I don't have enough data to answer this accurately based on the available syllabi regarding courses that *focus* on using AI tools. The provided context only details the policies for their use as an aid or their prohibition.</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The provided context does not explicitly identify courses that *focus* on using AI tools as a primary learning objective or method. However, several courses permit the use of AI tools under specific conditions for assignments or projects.
+Here are the courses where AI tools are permitted, which might align with your interest in using such tools:
+| Course   | AI Tool Usage Policy                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                </t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -4967,6 +5461,15 @@
 *   **Week 12-14:** Large Language Models (Basics, with Search Engines, for Ranking and Recommendation) [Source 2]</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>In the second half of CSCE 670, the course covers the following specific information retrieval algorithms and models:
+*   **Week 8:** word2vec; Neural Ranking [Source 2]
+*   **Week 10:** Transformer; BERT-Based Ranking [Source 2]
+*   **Week 11:** Neural Collaborative Filtering; Sequential Recommendation [Source 2]
+*   **Week 12-14:** Large Language Models (Basics, with Search Engines, for Ranking and Recommendation) [Source 2]</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5041,6 +5544,12 @@
         </is>
       </c>
       <c r="Q37" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 633 covers regularization techniques, as indicated by the "Logistic Regression &amp; Regularization" module in the course schedule [3].
+The provided context does not explicitly mention whether ensemble methods are covered [1, 3].</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
         <is>
           <t>Yes, CSCE 633 covers regularization techniques, as indicated by the "Logistic Regression &amp; Regularization" module in the course schedule [3].
 The provided context does not explicitly mention whether ensemble methods are covered [1, 3].</t>
@@ -5148,6 +5657,16 @@
 *   **Week 6:** Contextualized Representations, Pre-Training, Large Language Models [Source 1]</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 638 covers deep learning architectures including Transformers and Attention mechanisms [Source 1].
+The course schedule includes the following topics:
+*   **Week 3:** Convolutional Neural Network, Recurrent Neural Network
+*   **Week 4:** Sequence-to-Sequence, Attention
+*   **Week 5:** Transformers
+*   **Week 6:** Contextualized Representations, Pre-Training, Large Language Models [Source 1]</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -5215,6 +5734,11 @@
         </is>
       </c>
       <c r="Q39" t="inlineStr">
+        <is>
+          <t>I cannot find information about specific cryptographic concepts and protocols covered in CSCE 665 in the provided context [Source 1, Source 2, Source 3].</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>I cannot find information about specific cryptographic concepts and protocols covered in CSCE 665 in the provided context [Source 1, Source 2, Source 3].</t>
         </is>
@@ -5354,6 +5878,23 @@
 Homework assignments involve implementation and reports, requiring submissions to compile in Visual Studio 2022 [Source 3, 4]. Knowledge of UNIX and C programming is helpful but not required [Source 1].</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>CSCE 612: Applied Networks and Distributed Processing (Section 600) focuses on both network protocol implementation and distributed system design [Source 1].
+The course aims to:
+*   Mix fundamentals with programming and pragmatic engineering issues, including network architecture and principles of network engineering [Source 1].
+*   Apply principles of layered architecture to analyzing real networks, with lab exercises focusing on protocol understanding and programming [Source 1].
+*   Enable students to utilize operating-system sockets APIs, create efficient network applications, build multi-threaded decentralized frameworks, and develop protocols [Source 2].
+Key topics covered include:
+*   Sockets, threads, and synchronization [Source 3].
+*   Internet structure, topology, delay, and loss [Source 3].
+*   Application layer concepts such as HTTP, caching, cookies, FTP, email, and DNS [Source 3, 4].
+*   Transport layer topics like multiplexing, UDP, reliable data transfer (stop &amp; wait, Go-back-N, Selective Repeat), flow control, congestion control, and TCP modeling [Source 3, 4].
+*   Network layer concepts including switching, IP header, NAT, and routing protocols (link-state, distance vector, RIP, OSPF, BGP) [Source 4].
+*   Data-link layer topics such as error detection/correction, CSMA, Ethernet, hubs, and switches [Source 4].
+Homework assignments involve implementation and reports, requiring submissions to compile in Visual Studio 2022 [Source 3, 4]. Knowledge of UNIX and C programming is helpful but not required [Source 1].</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -5450,6 +5991,15 @@
         </is>
       </c>
       <c r="Q41" t="inlineStr">
+        <is>
+          <t>For CSCE 670, the final grade is weighted as follows:
+*   **Homework**: 30% (five programming assignments) [Source 1]
+*   **Quizzes**: 20% (four brief in-class quizzes) [Source 1]
+*   **Final Exam**: 30% [Source 1]
+*   **Group Project**: 20% [Source 1]</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
         <is>
           <t>For CSCE 670, the final grade is weighted as follows:
 *   **Homework**: 30% (five programming assignments) [Source 1]
@@ -5593,6 +6143,20 @@
 The programming assignments contribute 400 points to the final grade [3].</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>CSCE 611 includes a series of design and programming assignments, referred to as Machine Problems (MPs), that guide students through designing and developing a simple operating system [3, 1]. There are 7 Machine Problems assigned throughout the semester [4, 6].
+These assignments cover various aspects of operating systems, including:
+*   **MP1:** Project setup, introduction to OS concepts, architectural support, OS structures, system calls, and interrupt/exception handling on the x86 architecture [4].
+*   **MP2:** Memory management, including allocation, address spaces, paging, advanced paging, TLB, segmentation, and virtual memory mechanisms [4].
+*   **MP3:** Page replacement policies and an introduction to concurrency and scheduling [4, 6].
+*   **MP4:** Thread dispatching on the x86, kernel vs. user-level threads, and event-based concurrency [6].
+*   **MP5:** Software and hardware solutions to the critical section problem, concurrent data structures, and atomic transactions [6].
+*   **MP6:** I/O management, device drivers, disks, RAID, flash memory, and file systems (including UNIX file systems) [6].
+*   **MP7:** Journaled and log-based file systems, and virtualization mechanisms including memory virtualization [6].
+The programming assignments contribute 400 points to the final grade [3].</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -5665,6 +6229,11 @@
           <t>For CSCE 633, no late assignments will be accepted. Late assignments are defined as any deliverables submitted after the established deadline [Source 1]. Work submitted as makeup for an excused absence is exempt from this policy [Source 1].</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>For CSCE 633, no late assignments will be accepted. Late assignments are defined as any deliverables submitted after the established deadline [Source 1]. Work submitted as makeup for an excused absence is exempt from this policy [Source 1].</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -5737,6 +6306,11 @@
           <t>I cannot find that information in the provided context. The prerequisites listed for CSCE 633 are CSCE 420 or CSCE 625 [Source 1].</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>I cannot find that information in the provided context. The prerequisites listed for CSCE 633 are CSCE 420 or CSCE 625 [Source 1].</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -5814,6 +6388,11 @@
           <t>Yes, CSCE 611 has an explicit policy regarding the use of AI tools or generative AI for assignments and exams. Students are prohibited from using any part (code, text, figures, etc.) developed by others, including AI, for programming assignments and homework. This means students should not submit or make use of AI-generated solutions [Source 1]. For exams, AI tools are listed as disallowed sources of information [Source 2].</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Yes, CSCE 611 has an explicit policy regarding the use of AI tools or generative AI for assignments and exams. Students are prohibited from using any part (code, text, figures, etc.) developed by others, including AI, for programming assignments and homework. This means students should not submit or make use of AI-generated solutions [Source 1]. For exams, AI tools are listed as disallowed sources of information [Source 2].</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -5884,6 +6463,413 @@
       <c r="Q46" t="inlineStr">
         <is>
           <t>For CSCE 612, all homework submissions must compile in Visual Studio 2022 in both debug and release mode [Source 3]. Knowledge of UNIX and C programming is helpful but not required [Source 1].</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>For CSCE 612, all homework submissions must compile in Visual Studio 2022 in both debug and release mode [Source 3]. Knowledge of UNIX and C programming is helpful but not required [Source 1].</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Is CSCE 638 or CSCE 670 more math-heavy, and what does each course primarily cover?</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CSCE 638 (Machine Learning) is slightly more math-heavy, with a stronger emphasis on linear algebra, probability theory, and mathematical optimization. CSCE 670 (Information Storage and Retrieval) focuses more on information retrieval systems and applications. Both courses involve machine learning concepts.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CSCE 638, CSCE 670</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>DIFFICULTY</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>| Course | Grading | Workload | Prerequisites |
+|---|---|---|---|
+| CSCE 670 | Not found | Homeworks, Quizzes, Research Project [Source 4, 5] | CSCE 310 or CSCE 603 or approval of instructor; graduate classification [Source 1, 3] |
+| CSCE 638 | Not found | Not found | Not found |
+## Detailed Comparison
+Regarding whether CSCE 638 or CSCE 670 is more math-heavy, the provided context does not explicitly state the mathematical intensity of either course. However, based on the topics and descriptions:
+**CSCE 670**
+The course covers "fundamental data structures and algorithms of information storage and retrieval systems" and "techniques to design and evaluate complete retrieval systems, including cover of algorithms for indexing, compressing, and querying very large collections" [Source 1]. Specific topics include "TF-IDF; Vector Space Model; BM25," "Link Analysis" (e.g., PageRank), "Learning to Rank," "Recommender Systems" (e.g., Matrix Factorization), "word2vec; Neural Ranking," "Transformer; BERT-Based Ranking," and "Large Language Models" [Source 3, 5]. These topics involve significant mathematical and algorithmic foundations, such as linear algebra, probability, and optimization. The prerequisites include CSCE 310 or CSCE 603, which are typically courses in data structures and algorithms [Source 1, 3].
+**CSCE 638**
+This course focuses on "Natural Language Processing (NLP) fundamentals including language models, automatic syntactic processing and semantic understanding" [Source 2]. NLP, by nature, relies heavily on statistical methods, probability, and machine learning algorithms. While the context for CSCE 638 does not list as many specific mathematically-oriented algorithms as CSCE 670, the underlying concepts of language models and semantic understanding are mathematically intensive.
+Both fields are mathematically grounded. However, CSCE 670's description and topic list provide more explicit examples of specific algorithms and models (e.g., Vector Space Model, BM25, Matrix Factorization, PageRank, Neural Ranking) that are known to involve detailed mathematical underpinnings.
+### Course Overview
+**CSCE 670**: This course focuses on Information Storage and Retrieval, covering the representation, storage, and access to very large multimedia document collections. It delves into fundamental data structures and algorithms for information storage and retrieval systems, techniques to design and evaluate complete retrieval systems, and algorithms for indexing, compressing, and querying large collections. It also covers web search, recommender systems, and recent research in neural models and Large Language Models [Source 1, 3, 5].
+**CSCE 638**: This course focuses on Natural Language Processing (NLP) fundamentals. It covers language models, automatic syntactic processing, semantic understanding, and introduces major NLP applications such as information extraction, machine translation, text summarization, dialogue systems, and sentiment analysis [Source 2].
+### Prerequisites
+**CSCE 670**: Prerequisites include CSCE 310 or CSCE 603 or approval of the instructor, along with graduate classification [Source 1, 3].
+**CSCE 638**: Not found.
+### Learning Outcomes
+**CSCE 670**: Upon completion, learners will be able to:
+*   Define and explain key concepts and models relevant to web search (e.g., text indexing, retrieval models, evaluation, Web crawling, PageRank, learning to rank).
+*   Define and explain key concepts and models relevant to recommender systems (e.g., collaborative filtering, matrix factorization, evaluation, implicit recommendation).
+*   Design, implement, and evaluate core algorithms for fully functional web search and recommendation systems.
+*   Identify salient features and apply recent research results in web search and recommender systems, including adversarial information retrieval and neural models [Source 3].
+**CSCE 638**: Upon completion, learners will be able to:
+*   Identify and explain the fundamental concepts and models for natural language processing.
+*   Be aware of recent trends in natural language processing research [Source 2].
+### Topics
+**CSCE 670**: The course schedule includes topics such as Course Overview, Boolean Retrieval, TF-IDF, Vector Space Model, BM25, Link Analysis, Evaluation of Search Engines, Learning to Rank, Recommender Systems (Content-Based, Collaborative Filtering, Matrix Factorization, Bayesian Personalized Ranking), word2vec, Neural Ranking, Transformer, BERT-Based Ranking, Neural Collaborative Filtering, Sequential Recommendation, Large Language Models Basics, Large Language Models with Search Engines, and Large Language Models for Ranking and Recommendation [Source 5].
+**CSCE 638**: The course covers Natural Language Processing (NLP) fundamentals including language models, automatic syntactic processing, semantic understanding, and major NLP applications such as information extraction, machine translation, text summarization, dialogue systems, and sentiment analysis [Source 2].
+### Materials
+**CSCE 670**: An optional textbook is "Mining of Massive Datasets" by Jure Leskovec, Anand Rajaraman, and Jeffrey D. Ullman (2014) [Source 3].
+**CSCE 638**: Not found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>48</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>How does the grading structure of CSCE 312 compare to CSCE 313? Which course relies more on projects versus exams?</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Both CSCE 312 and CSCE 313 include exams and projects. CSCE 312 is more weighted toward projects relative to exams/quizzes, while CSCE 313 places relatively greater emphasis on exams.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>CSCE 312, CSCE 313</t>
+        </is>
+      </c>
+      <c r="K48" t="b">
+        <v>0</v>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>No relevant documents found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>49</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Between CSCE 221 and CSCE 222, which has the heavier homework load?</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CSCE 221 generally has the heavier homework load. CSCE 222 depends more on exams. The difference is not extreme.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>CSCE 221, CSCE 222</t>
+        </is>
+      </c>
+      <c r="K49" t="b">
+        <v>0</v>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>50</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>What CSCE graduate courses involve machine learning or artificial intelligence?</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CSCE 638 (Machine Learning), CSCE 636 (Deep Learning), and CSCE 625 (Artificial Intelligence) explicitly focus on ML/AI. Many other CSCE graduate courses also incorporate elements of machine learning or artificial intelligence.</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ACADEMIC</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Several CSCE graduate courses involve machine learning or artificial intelligence:
+*   **CSCE 726: Large-scale Optimization for Machine Learning**
+    *   This course focuses on fundamental optimization algorithms and their analysis for solving machine learning problems, including deterministic and stochastic gradient-based algorithms. It emphasizes the role of large-scale optimization in ML and AI [Source 3, 9]. Students are expected to have basic knowledge of machine learning and deep learning [Source 1, 9].
+*   **CSCE 633: Machine Learning**
+    *   This course is the study of self-modifying computer systems that can acquire new knowledge and improve their performance. It surveys machine learning techniques such as induction from examples, conceptual clustering, explanation-based learning, exemplar learning, analogy, discovery, and genetic algorithms [Source 4].
+*   **CSCE 635: AI Robotics**
+    *   This course provides an introduction and survey of artificial intelligence methods for mobile robots, focusing on biological and cognitive principles. It covers core concepts in robotic autonomy, including state estimation, planning, control, and decision-making under uncertainty [Source 8].
+*   **CSCE 670: Information Retrieval and Recommender Systems**
+    *   This course involves topics like text indexing, retrieval models, evaluation, Web crawling, link-based algorithms, and learning to rank, as well as recommender systems, collaborative filtering, and matrix factorization. It also mentions applying recent research results, including neural models of retrieval and recommendation [Source 6].
+*   **CSCE 676: Data Mining and Analysis**
+    *   This course provides a broad overview of data mining, integrating related concepts from machine learning and statistics. It covers exploratory data analysis, pattern mining, clustering, and classification, with applications to scientific and online data [Source 10].
+*   **CSCE 679: Data Visualization**
+    *   While primarily focused on visualization, this course discusses the role of data visualization in Explainable AI and involves programming in Python for data and AI [Source 7].
+*   **CSCE 624: Sketch Recognition**
+    *   This course emphasizes how systems interpret sketches and how recognition algorithms behave in real-world settings. It mentions that familiarity with basic machine learning or artificial intelligence concepts can be helpful [Source 5].</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>51</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>What CSCE courses cover formal methods or theoretical computer science topics?</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CSCE 627 (Theory of Computation), CSCE 411 (Design and Analysis of Algorithms), CSCE 222 (Discrete Structures for Computing), and CSCE 221 cover formal methods or theoretical computer science concepts.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ACADEMIC</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>The principle underlying "formal methods" and "theoretical computer science" in an academic context involves the use of mathematical logic, discrete mathematics, and abstract models to specify, develop, and verify hardware and software systems, or to analyze the fundamental capabilities and limitations of computation. This includes topics like algorithm analysis, complexity theory, computability, and formal language theory.
+Based on the provided context, the following CSCE courses cover topics related to formal methods or theoretical computer science:
+*   **CSCE 629: Analysis of Algorithms**
+    *   **Academic Dimension:** This course focuses on "Concrete algorithm design and analysis; abstract models to analyze the complexity of problems; NP-Completeness; approximation and probabilistic algorithms" [Source 2].
+    *   **Learning Outcomes:** Students will learn to "Explain a variety of fundamental algorithms and algorithmic techniques," "Select the most appropriate algorithm to solve a given problem," "Analyze the correctness, runtime, and space complexity of an algorithm," "Design new algorithms and modify existing ones using techniques discussed in class," and "Recognize when a problem is likely intractable (has no efficient algorithm) and be able to prove this by showing undecidability or NP-hardness" [Source 2, 6]. These outcomes directly align with theoretical computer science, particularly complexity theory and algorithm analysis.
+*   **CSCE 669: Computational Optimization**
+    *   **Academic Dimension:** This course delves into "Combinatorial theory of polytopes as a tool for the solution of combinatorial optimization problems; applications to max flow, matching and matroids; geometric interpretation of the results indicating the profound role that polyhedral combinatorics play in the design and complexity of approximation algorithms" [Source 10].
+    *   **Learning Outcomes:** Students are expected to "Master basic theories and techniques in the current research in computational optimization" and "apply theories and techniques studied in the course to solve real-world problems" [Source 10]. The emphasis on "combinatorial theory," "polyhedral combinatorics," and "complexity of approximation algorithms" places this course firmly within theoretical computer science and formal methods for optimization.
+While CSCE 633 (Machine Learning) mentions the ability to "formalize the fundamental techniques and methods of machine learning" [Source 3], its primary focus as described is on surveying machine learning techniques rather than the foundational mathematical logic or abstract models typically associated with a dedicated formal methods or theoretical computer science course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>52</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Are there CSCE courses focused on parallel or distributed computing?</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Parallel and distributed computing is a specialized topic in the CSCE curriculum. CSCE 735 (Distributed and Parallel Computing) is the primary graduate course, though it may not be available in the current syllabus database. Other courses may touch on these topics tangentially.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ACADEMIC</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Yes, there are CSCE courses that focus on parallel or distributed computing.
+The relevant principle here is **distributed systems** and **parallel computing**, which involve coordinating multiple computational units to achieve a common goal, often for performance or fault tolerance.
+Based on the provided syllabi, the following courses cover aspects of parallel or distributed computing:
+*   **CSCE 612: Applied Networks and Distributed Processing**
+    *   **Principle**: This course directly addresses "Distributed Processing" and focuses on applying principles of layered architecture to analyzing real networks [Source 1].
+    *   **Academic Content**: Students will learn to create efficient network applications and build multi-threaded decentralized frameworks [Source 4].
+*   **CSCE 611: Operating Systems**
+    *   **Principle**: This course provides an overview of operating systems, including understanding fundamental approaches to virtualization and what it takes to build a distributed system [Source 3]. It also covers concurrency and synchronization [Source 3, 6].
+    *   **Academic Content**: Topics include evaluating and comparing various forms of concurrency and synchronization mechanisms, and understanding thread dispatching [Source 3, 6].
+*   **CSCE 614: Computer Architecture**
+    *   **Principle**: This course reviews computer architecture with an emphasis on microprocessor design, including parallel computer structures and concurrent computation [Source 2].
+    *   **Academic Content**: It covers pipeline computers, vectorization methods, array processors, and multiprocessor architectures and programming [Source 2]. The schedule also lists topics like ILP (Instruction-Level Parallelism), SIMD (Single Instruction, Multiple Data), and TLP (Thread-Level Parallelism) [Source 8].</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>53</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>What should I take after completing CSCE 638?</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Good follow-up courses after CSCE 638 (Machine Learning) include CSCE 670 (Information Storage and Retrieval) and CSCE 753.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>CSCE 638</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>CSCE 638</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>PLANNING</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Academic progression often involves building upon foundational knowledge or exploring related sub-disciplines. When direct prerequisites or recommended sequences are not explicitly stated, students can consider courses that share thematic elements or offer advanced applications of concepts learned in a prior course.
+Based on the provided syllabi, there is no explicit recommendation for a specific course to take immediately after CSCE 638. However, CSCE 638, "Natural Language Processing: Foundations and Techniques," covers "Large Language Models" as a key topic [Source 1, 3].
+Another course, CSCE 670, "Information Retrieval," also extensively covers "Large Language Models Basics," "Large Language Models with Search Engines," and "Large Language Models for Ranking and Recommendation" [Source 4]. This indicates a thematic overlap and suggests that CSCE 670 could be a relevant course for students interested in applying or further exploring Large Language Models within the context of information retrieval and recommender systems, building on the foundations established in CSCE 638.
+I don't have enough data to definitively recommend a specific next course based on the available syllabi, as no explicit academic progression or prerequisite relationships are provided for courses following CSCE 638.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>54</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>What courses pair well with CSCE 676?</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CSCE 670 pairs well with CSCE 676, as both involve information retrieval and data-intensive systems.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>CSCE 676</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>CSCE 676</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>PLANNING</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>CSCE 676 is cross-listed with ECEN 758 and STAT 639 [Source 1]. This means they are the same course, and the information provided for CSCE 676 applies to ECEN 758 and STAT 639.
+| Course | Grading | Workload | Prerequisites |
+|---|---|---|---|
+| CSCE 676 / ECEN 758 / STAT 639 | 10% Weekly Assessments, 50% Homework, 40% Individual Semester-Long Project [Source 3, 4] | Weekly assessments, weekly homework assignments, and a semester-long individual project with five deliverables [Source 4, 5] | Previous exposure to basic probability, statistics, algorithms, and data structures; ability to design/develop large programs and learn new software libraries [Source 1] |
+## Detailed Comparison
+### Course Overview
+**CSCE 676, ECEN 758, STAT 639**: This course provides a broad overview of data mining, integrating related concepts from machine learning and statistics. Topics include exploratory data analysis, pattern mining, clustering, and classification, with applications to scientific and online data. It is cross-listed with ECEN 758 and STAT 639 [Source 1].
+### Grading &amp; Workload
+**CSCE 676, ECEN 758, STAT 639**:
+*   **Grading**: The final grade is composed of 10% Weekly Assessments, 50% Homework, and 40% Individual Semester-Long Project [Source 3].
+    *   Weekly Assessments: Short quizzes (typically true/false, multiple choice) over the week's material, which can be taken multiple times with the highest score kept [Source 4].
+    *   Homework: Weekly assignments for the first twelve weeks (4% each) and a 13th homework (2%). These are Python notebooks with programming, written problems, and other questions. Students are required to use an AI-coding assistant. No prior Python exposure is expected, but rapid learning is required [Source 4].
+    *   Individual Semester-Long Project: A significant data mining project broken into five deliverables: Data Selection (Feb 3), Initial Research Question (Mar 5), Deep Dive (Apr 2), Project Showcase (week of Apr 20), and Final Deliverable (Apr 27) [Source 5, 2].
+*   **Late Work Policy**: Late homework is penalized 1% per hour after the deadline, up to a maximum of 48 hours, after which it receives a 0. For the Individual Semester-Long Project, students have five late days in total for the first three deliverables. The Project Showcase and Final Deliverable will not be accepted late [Source 5, 2].
+### Prerequisites
+**CSCE 676, ECEN 758, STAT 639**: Students are expected to have previous exposure to basic probability, statistics, algorithms, and data structures. They should also be able to design and develop large programs and learn new software libraries independently [Source 1].
+### Learning Outcomes
+**CSCE 676, ECEN 758, STAT 639**: Upon completion, learners will be able to:
+*   Define and explain key concepts and models in data mining and analysis, including data preparation, normalization, dimensionality reduction, and text mining [Source 3].
+*   Design, implement, and evaluate data mining algorithms (e.g., associate rules, clustering, anomaly detection) on modern scalable cloud computing platforms (e.g., Spark) [Source 3].
+*   Identify salient features and apply recent research results in data mining, including topics like graph mining and large-scale mining [Source 3].
+### Topics
+**CSCE 676, ECEN 758, STAT 639**: The course schedule includes: Course introduction, Frequent Itemset Mining, Graph Mining, Graph Mining and Large-Scale ML, Large-Scale ML, Clustering, Text Mining, Data Mining and Distributed Computing, Anomaly Detection, Graph Embeddings, Locality-Sensitive Hashing, Stream Mining, Hot Topics in Data Mining, Project Showcase, and Finalize Project Deliverables [Source 2].
+### Materials
+**CSCE 676, ECEN 758, STAT 639**: Required course readings will be drawn from various online textbooks, scholarly papers, and other resources. A key required textbook is "Mining of Massive Data Sets" by Jure Leskovec, Anand Rajaraman, and Jeffrey David Ullman (Cambridge University Press, 2020) [Source 3].</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>55</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>What's the weather in College Station today?</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>out_of_scope</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Howdy! I'm TamuBot, your Texas A&amp;M academic assistant. I can help you with questions about courses, syllabi, grading policies, schedules, and university policies. What would you like to know?</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>56</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Write me a Python script to sort a list of numbers</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>out_of_scope</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Howdy! I'm TamuBot, your Texas A&amp;M academic assistant. I can help you with questions about courses, syllabi, grading policies, schedules, and university policies. What would you like to know?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand golden set diversity
</commit_message>
<xml_diff>
--- a/tamu_data/evals/golden_sets/golden_20260411_v1.xlsx
+++ b/tamu_data/evals/golden_sets/golden_20260411_v1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6873,6 +6873,411 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>57</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>What should I take alongside CSCE 670 to build toward a research career in information retrieval?</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>CSCE 638 (NLP) pairs naturally with CSCE 670 as both deal with language and text processing. CSCE 633 (Machine Learning) is also a strong complement, providing the statistical foundations underlying modern IR systems.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>CSCE 670</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>CSCE 670</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>PLANNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>58</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Which CSCE grad courses allow or encourage using AI tools for assignments?</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Several CSCE grad courses explicitly permit or encourage AI tool usage, including CSCE 638, CSCE 670, CSCE 676, and CSCE 753, among others. Policies vary by course and assignment type — always check the specific syllabus.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>POLICY</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>59</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Which CSCE grad courses require buying a textbook?</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CSCE 676 explicitly requires a paid textbook: 'Mining of Massive Data Sets' by Leskovec, Rajaraman, and Ullman. Most other CSCE grad courses rely on free online readings and papers.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>CSCE 676</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>MATERIALS</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>MATERIALS</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>LOGISTICAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>60</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>What do I need before taking CSCE 629?</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Graduate classification is the only formal prerequisite for CSCE 629. However, the course assumes strong background knowledge in algorithms and complexity theory.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>CSCE 629</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>PREREQUISITES</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CSCE 629</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>PREREQUISITES</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>LOGISTICAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>61</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Which CSCE grad courses have the lightest prerequisites?</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Most CSCE graduate courses formally only require graduate classification. Courses like CSCE 676 and CSCE 670 are generally considered more accessible in terms of expected background, while others like CSCE 629 carry a steeper implied expectation despite the same formal requirement.</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>PREREQUISITES</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>PREREQUISITES</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>PLANNING</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>62</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Can I use ChatGPT to help write my assignments for CSCE 638?</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Yes. CSCE 638 explicitly allows the use of AI tools including ChatGPT for assignments.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>CSCE 638</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>CSCE 638</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>POLICY</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>63</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Which CSCE grad courses have the strictest AI policies?</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CSCE 629 and CSCE 752 both prohibit AI tools entirely. CSCE 633 has a partial restriction — AI is prohibited for some assignments but permitted for others.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>recursive</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>AI_POLICY</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>POLICY</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>64</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Compare the grading breakdown of CSCE 629, CSCE 633, and CSCE 670 — which is the most exam-heavy?</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>From least to most exam-heavy: CSCE 670 relies primarily on projects and papers with no traditional exams. CSCE 633 has a moderate exam component. CSCE 629 is the most exam-heavy of the three.</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>GRADING</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>CSCE 629|CSCE 633|CSCE 670</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>GRADING</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>COMPARISON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>65</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>What time does the CSCE department office open?</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>out_of_scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>66</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Do any CSCE grad courses have in-person attendance requirements?</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Some CSCE grad courses specify attendance expectations in their syllabi. Students should review each course's syllabus directly for specific attendance policies.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>semantic_general</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>SCHEDULE</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>SCHEDULE</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>LOGISTICAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>67</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>When is the midterm exam for CSCE 629?</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>The midterm exam for CSCE 629 is scheduled for October 6th.</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>hybrid_course</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>CSCE 629</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>SCHEDULE</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>CSCE 629</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>SCHEDULE</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>LOGISTICAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>